<commit_message>
add 2 set setlist
</commit_message>
<xml_diff>
--- a/setlists/Stove Up.xlsx
+++ b/setlists/Stove Up.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Stove Up" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Stove Up 2 sets" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="200">
   <si>
     <t xml:space="preserve">Song</t>
   </si>
@@ -623,6 +624,18 @@
   </si>
   <si>
     <t xml:space="preserve">Champ Supernova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semi-Charmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">--- Set 2 ---</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- All For You</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blitzkreig</t>
   </si>
 </sst>
 </file>
@@ -683,12 +696,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <i val="true"/>
       <sz val="10"/>
       <color theme="1"/>
@@ -699,6 +706,14 @@
     <font>
       <i val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -771,7 +786,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -844,7 +859,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -860,12 +875,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2344,7 +2363,6 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
       <c r="C17" s="23"/>
     </row>
     <row r="18" customFormat="false" ht="35.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2361,4 +2379,191 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="33.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.64"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="20"/>
+    </row>
+    <row r="15" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="15"/>
+    </row>
+    <row r="17" customFormat="false" ht="33.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="15"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>